<commit_message>
help formulae sheet is ready
</commit_message>
<xml_diff>
--- a/skillbox/2.6 Case Filled.xlsx
+++ b/skillbox/2.6 Case Filled.xlsx
@@ -20,7 +20,7 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="Z3xi6G1BNgeSwbgbfDU4Hn2WKVhro2ChGy2Be3b4kcw="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="" roundtripDataChecksum="Z3xi6G1BNgeSwbgbfDU4Hn2WKVhro2ChGy2Be3b4kcw="/>
     </ext>
   </extLst>
 </workbook>
@@ -1424,7 +1424,7 @@
       <c r="D41" s="15">
         <v>-351394</v>
       </c>
-      <c r="F41" s="20" t="s">
+      <c r="F41" t="s">
         <v>31</v>
       </c>
       <c r="G41" s="19">
@@ -1482,7 +1482,7 @@
       <c r="D43" s="8">
         <v>-85357</v>
       </c>
-      <c r="F43" s="20" t="s">
+      <c r="F43" t="s">
         <v>35</v>
       </c>
       <c r="G43" s="19">

</xml_diff>